<commit_message>
Normalizar finales de línea. Reporte ventas cuero junio. Reporte histórico joyería a junio 2026. Comienzo de preparación de datos para presupuestos y gastos junio 2026
</commit_message>
<xml_diff>
--- a/Reporte_ventas/Colores excel para materiales.xlsx
+++ b/Reporte_ventas/Colores excel para materiales.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\Valeria\Reportes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maval\Documents\Vale laburo\Castelli\Reportes\Reporte_ventas\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6930"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9192"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="19">
   <si>
     <t>ROJO</t>
   </si>
@@ -78,6 +78,9 @@
   </si>
   <si>
     <t>OLIVE</t>
+  </si>
+  <si>
+    <t>HEREFORD/TABACO</t>
   </si>
 </sst>
 </file>
@@ -395,18 +398,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D19"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:D20"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -420,7 +423,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -434,7 +437,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -448,7 +451,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -462,7 +465,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -476,7 +479,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -490,7 +493,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -504,7 +507,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -518,7 +521,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -532,7 +535,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -546,7 +549,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -560,7 +563,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>2</v>
       </c>
@@ -574,7 +577,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -588,7 +591,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -602,7 +605,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -616,7 +619,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -630,7 +633,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>17</v>
       </c>
@@ -642,6 +645,20 @@
       </c>
       <c r="D19">
         <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>18</v>
+      </c>
+      <c r="B20">
+        <v>89</v>
+      </c>
+      <c r="C20">
+        <v>59</v>
+      </c>
+      <c r="D20">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>